<commit_message>
feat: add proceeds sensitivity (multiple-based) + traceable Q1 anchor; address final review
</commit_message>
<xml_diff>
--- a/examples/foxfactory/output/foxf-forecast.xlsx
+++ b/examples/foxfactory/output/foxf-forecast.xlsx
@@ -10,7 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast (monthly)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segments FY2026" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segments FY2027" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Divestiture" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Divestiture (timing)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Divestiture (price)" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2157,4 +2158,104 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>proceeds_case</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>proceeds</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>two_yr_fcf</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>net_debt_to_ebitda</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>At cost (~$567M paid)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>567194000</v>
+      </c>
+      <c r="C2" t="n">
+        <v>200786654.4493412</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-0.2489865514784787</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Default markdown</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>300000000</v>
+      </c>
+      <c r="C3" t="n">
+        <v>184113748.8493412</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.274921104645322</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>8x EBITDA</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>600000000</v>
+      </c>
+      <c r="C4" t="n">
+        <v>202833748.8493412</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-0.4360914811056313</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>12x EBITDA</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>900000000</v>
+      </c>
+      <c r="C5" t="n">
+        <v>221553748.8493412</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-2.147104066856585</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: regenerate Fox Factory epoch artifacts after improvement-clamp fix
Epoch foxf-fy2025-001: adjusted_ebitda_error improvement clamped from -18.85
to -1.0; weighted_improvement 0.056 (was -5.30); objective_gain 0.055 (was
-5.30); status proposed (was discarded). Epoch foxf-fy2025-002 numbers
unchanged. Artifacts generated from code via run_foxf.py, not hand-edited.
</commit_message>
<xml_diff>
--- a/examples/foxfactory/output/foxf-forecast.xlsx
+++ b/examples/foxfactory/output/foxf-forecast.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical holdout" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast (monthly)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segments FY2026" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segments FY2027" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Divestiture (timing)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Divestiture (price)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Historical holdout" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Forecast (monthly)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Segments FY2026" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Segments FY2027" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Divestiture (timing)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Divestiture (price)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,16 +25,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -45,7 +42,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -53,24 +50,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,47 +426,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>epoch</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>hypothesis</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>metric</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>champion_error</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>challenger_error</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>error_improvement</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>objective_gain</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>promotion_eligible</t>
         </is>
@@ -494,7 +480,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>discarded</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -517,10 +503,10 @@
         <v>0.02394056924149505</v>
       </c>
       <c r="H2" t="n">
-        <v>-5.299602720263328</v>
+        <v>0.05496885872055847</v>
       </c>
       <c r="I2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -531,7 +517,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>discarded</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -554,10 +540,10 @@
         <v>0.0427810249352692</v>
       </c>
       <c r="H3" t="n">
-        <v>-5.299602720263328</v>
+        <v>0.05496885872055847</v>
       </c>
       <c r="I3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -568,7 +554,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>discarded</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -591,10 +577,10 @@
         <v>-0.1936685880242516</v>
       </c>
       <c r="H4" t="n">
-        <v>-5.299602720263328</v>
+        <v>0.05496885872055847</v>
       </c>
       <c r="I4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -605,7 +591,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>discarded</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -628,10 +614,10 @@
         <v>0.006896152791465091</v>
       </c>
       <c r="H5" t="n">
-        <v>-5.299602720263328</v>
+        <v>0.05496885872055847</v>
       </c>
       <c r="I5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -797,94 +783,94 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>revenue</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>cogs</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>gross_profit</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>opex</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ebitda</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>da</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>interest</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>pretax_income</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>tax</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>net_income</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>wc_cash_impact</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>operating_cash_flow</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>capex</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>principal</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>free_cash_flow</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>change_in_cash</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>ending_cash</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
         <v>46023</v>
       </c>
       <c r="B2" t="n">
@@ -940,7 +926,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="1" t="n">
         <v>46054</v>
       </c>
       <c r="B3" t="n">
@@ -996,7 +982,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>46082</v>
       </c>
       <c r="B4" t="n">
@@ -1052,7 +1038,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>46113</v>
       </c>
       <c r="B5" t="n">
@@ -1108,7 +1094,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="1" t="n">
         <v>46143</v>
       </c>
       <c r="B6" t="n">
@@ -1164,7 +1150,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="B7" t="n">
@@ -1220,7 +1206,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="1" t="n">
         <v>46204</v>
       </c>
       <c r="B8" t="n">
@@ -1276,7 +1262,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="1" t="n">
         <v>46235</v>
       </c>
       <c r="B9" t="n">
@@ -1332,7 +1318,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="1" t="n">
         <v>46266</v>
       </c>
       <c r="B10" t="n">
@@ -1388,7 +1374,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="1" t="n">
         <v>46296</v>
       </c>
       <c r="B11" t="n">
@@ -1444,7 +1430,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="1" t="n">
         <v>46327</v>
       </c>
       <c r="B12" t="n">
@@ -1500,7 +1486,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="1" t="n">
         <v>46357</v>
       </c>
       <c r="B13" t="n">
@@ -1556,7 +1542,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="1" t="n">
         <v>46388</v>
       </c>
       <c r="B14" t="n">
@@ -1612,7 +1598,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="1" t="n">
         <v>46419</v>
       </c>
       <c r="B15" t="n">
@@ -1668,7 +1654,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="1" t="n">
         <v>46447</v>
       </c>
       <c r="B16" t="n">
@@ -1724,7 +1710,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="1" t="n">
         <v>46478</v>
       </c>
       <c r="B17" t="n">
@@ -1780,7 +1766,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="1" t="n">
         <v>46508</v>
       </c>
       <c r="B18" t="n">
@@ -1836,7 +1822,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="1" t="n">
         <v>46539</v>
       </c>
       <c r="B19" t="n">
@@ -1892,7 +1878,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="1" t="n">
         <v>46569</v>
       </c>
       <c r="B20" t="n">
@@ -1948,7 +1934,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="1" t="n">
         <v>46600</v>
       </c>
       <c r="B21" t="n">
@@ -2004,7 +1990,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="1" t="n">
         <v>46631</v>
       </c>
       <c r="B22" t="n">
@@ -2060,7 +2046,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="1" t="n">
         <v>46661</v>
       </c>
       <c r="B23" t="n">
@@ -2116,7 +2102,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="1" t="n">
         <v>46692</v>
       </c>
       <c r="B24" t="n">
@@ -2172,7 +2158,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" s="1" t="n">
         <v>46722</v>
       </c>
       <c r="B25" t="n">
@@ -2242,29 +2228,29 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>net_sales</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>adjusted_ebitda</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ebitda_margin</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>PVG</t>
         </is>
@@ -2280,7 +2266,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>AAG</t>
         </is>
@@ -2296,7 +2282,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>SSG</t>
         </is>
@@ -2326,29 +2312,29 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>net_sales</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>adjusted_ebitda</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ebitda_margin</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>PVG</t>
         </is>
@@ -2364,7 +2350,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>AAG</t>
         </is>
@@ -2380,7 +2366,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>SSG</t>
         </is>
@@ -2410,29 +2396,29 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>scenario</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>sale_month</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>two_yr_fcf</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>net_debt_to_ebitda</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Hold Marucci</t>
         </is>
@@ -2450,7 +2436,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Sell at 6mo</t>
         </is>
@@ -2466,7 +2452,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Sell at 12mo</t>
         </is>
@@ -2482,7 +2468,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Sell at 18mo</t>
         </is>
@@ -2498,7 +2484,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Sell at 24mo</t>
         </is>
@@ -2528,29 +2514,29 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>proceeds_case</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>proceeds</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>two_yr_fcf</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>net_debt_to_ebitda</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>At cost (~$567M paid)</t>
         </is>
@@ -2566,7 +2552,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Default markdown</t>
         </is>
@@ -2582,7 +2568,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>8x EBITDA</t>
         </is>
@@ -2598,7 +2584,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>12x EBITDA</t>
         </is>

</xml_diff>

<commit_message>
fix: add max_metric_regression hard guard so the clamp cannot launder a catastrophic single-metric regression; Fox epoch 001 discarded for the principled reason
</commit_message>
<xml_diff>
--- a/examples/foxfactory/output/foxf-forecast.xlsx
+++ b/examples/foxfactory/output/foxf-forecast.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Historical holdout" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Forecast (monthly)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Segments FY2026" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Segments FY2027" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Divestiture (timing)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Divestiture (price)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical holdout" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast (monthly)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segments FY2026" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segments FY2027" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Divestiture (timing)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Divestiture (price)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,13 +25,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -42,7 +45,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -50,13 +53,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,47 +440,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>epoch</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>hypothesis</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>metric</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>champion_error</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>challenger_error</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>error_improvement</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>objective_gain</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>promotion_eligible</t>
         </is>
@@ -480,7 +494,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -506,7 +520,7 @@
         <v>0.05496885872055847</v>
       </c>
       <c r="I2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -517,7 +531,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -543,7 +557,7 @@
         <v>0.05496885872055847</v>
       </c>
       <c r="I3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -554,7 +568,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -580,7 +594,7 @@
         <v>0.05496885872055847</v>
       </c>
       <c r="I4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -591,7 +605,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -617,7 +631,7 @@
         <v>0.05496885872055847</v>
       </c>
       <c r="I5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -783,94 +797,94 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>revenue</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>cogs</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>gross_profit</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>opex</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>ebitda</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>da</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>interest</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>pretax_income</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>tax</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>net_income</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>wc_cash_impact</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>operating_cash_flow</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>capex</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>principal</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>free_cash_flow</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>change_in_cash</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>ending_cash</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>46023</v>
       </c>
       <c r="B2" t="n">
@@ -926,7 +940,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>46054</v>
       </c>
       <c r="B3" t="n">
@@ -982,7 +996,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>46082</v>
       </c>
       <c r="B4" t="n">
@@ -1038,7 +1052,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>46113</v>
       </c>
       <c r="B5" t="n">
@@ -1094,7 +1108,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>46143</v>
       </c>
       <c r="B6" t="n">
@@ -1150,7 +1164,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="B7" t="n">
@@ -1206,7 +1220,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>46204</v>
       </c>
       <c r="B8" t="n">
@@ -1262,7 +1276,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>46235</v>
       </c>
       <c r="B9" t="n">
@@ -1318,7 +1332,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="2" t="n">
         <v>46266</v>
       </c>
       <c r="B10" t="n">
@@ -1374,7 +1388,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" s="2" t="n">
         <v>46296</v>
       </c>
       <c r="B11" t="n">
@@ -1430,7 +1444,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" s="2" t="n">
         <v>46327</v>
       </c>
       <c r="B12" t="n">
@@ -1486,7 +1500,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" s="2" t="n">
         <v>46357</v>
       </c>
       <c r="B13" t="n">
@@ -1542,7 +1556,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" s="2" t="n">
         <v>46388</v>
       </c>
       <c r="B14" t="n">
@@ -1598,7 +1612,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" s="2" t="n">
         <v>46419</v>
       </c>
       <c r="B15" t="n">
@@ -1654,7 +1668,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" s="2" t="n">
         <v>46447</v>
       </c>
       <c r="B16" t="n">
@@ -1710,7 +1724,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" s="2" t="n">
         <v>46478</v>
       </c>
       <c r="B17" t="n">
@@ -1766,7 +1780,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="2" t="n">
         <v>46508</v>
       </c>
       <c r="B18" t="n">
@@ -1822,7 +1836,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" s="2" t="n">
         <v>46539</v>
       </c>
       <c r="B19" t="n">
@@ -1878,7 +1892,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" s="2" t="n">
         <v>46569</v>
       </c>
       <c r="B20" t="n">
@@ -1934,7 +1948,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" s="2" t="n">
         <v>46600</v>
       </c>
       <c r="B21" t="n">
@@ -1990,7 +2004,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" s="2" t="n">
         <v>46631</v>
       </c>
       <c r="B22" t="n">
@@ -2046,7 +2060,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" s="2" t="n">
         <v>46661</v>
       </c>
       <c r="B23" t="n">
@@ -2102,7 +2116,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" s="2" t="n">
         <v>46692</v>
       </c>
       <c r="B24" t="n">
@@ -2158,7 +2172,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" s="2" t="n">
         <v>46722</v>
       </c>
       <c r="B25" t="n">
@@ -2228,29 +2242,29 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>net_sales</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>adjusted_ebitda</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ebitda_margin</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>PVG</t>
         </is>
@@ -2266,7 +2280,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>AAG</t>
         </is>
@@ -2282,7 +2296,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>SSG</t>
         </is>
@@ -2312,29 +2326,29 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>net_sales</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>adjusted_ebitda</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ebitda_margin</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>PVG</t>
         </is>
@@ -2350,7 +2364,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>AAG</t>
         </is>
@@ -2366,7 +2380,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>SSG</t>
         </is>
@@ -2396,29 +2410,29 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>scenario</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>sale_month</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>two_yr_fcf</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>net_debt_to_ebitda</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Hold Marucci</t>
         </is>
@@ -2436,7 +2450,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Sell at 6mo</t>
         </is>
@@ -2452,7 +2466,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Sell at 12mo</t>
         </is>
@@ -2468,7 +2482,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Sell at 18mo</t>
         </is>
@@ -2484,7 +2498,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>Sell at 24mo</t>
         </is>
@@ -2514,29 +2528,29 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>proceeds_case</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>proceeds</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>two_yr_fcf</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>net_debt_to_ebitda</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>At cost (~$567M paid)</t>
         </is>
@@ -2552,7 +2566,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Default markdown</t>
         </is>
@@ -2568,7 +2582,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>8x EBITDA</t>
         </is>
@@ -2584,7 +2598,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>12x EBITDA</t>
         </is>

</xml_diff>